<commit_message>
上新 JayESims XOXOGossipGirlRichTeaRumors 绯闻女孩：八卦社交名流公司
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -15,12 +15,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * -#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="_ \¥* #,##0.00_ ;_ \¥* -#,##0.00_ ;_ \¥* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * -#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="168" formatCode="_ \¥* #,##0_ ;_ \¥* -#,##0_ ;_ \¥* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -599,7 +600,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -679,6 +680,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0"/>
@@ -1022,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="19" min="1" max="1"/>
@@ -4018,6 +4028,68 @@
       </c>
       <c r="N46" s="21" t="n">
         <v>46276</v>
+      </c>
+    </row>
+    <row r="47" ht="36" customHeight="1" s="26">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B47" s="28" t="inlineStr">
+        <is>
+          <t>XOXOGossipGirlRichTeaRumors</t>
+        </is>
+      </c>
+      <c r="C47" s="28" t="inlineStr">
+        <is>
+          <t>绯闻女孩：八卦社交名流公司</t>
+        </is>
+      </c>
+      <c r="D47" s="28" t="inlineStr">
+        <is>
+          <t>JayESims</t>
+        </is>
+      </c>
+      <c r="E47" s="28" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/JayESims</t>
+        </is>
+      </c>
+      <c r="F47" s="28" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/JayESims/posts/jayesims-x-jaye-139755723</t>
+        </is>
+      </c>
+      <c r="G47" s="29" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H47" s="29" t="n">
+        <v>46279</v>
+      </c>
+      <c r="I47" s="27" t="inlineStr">
+        <is>
+          <t>XML 注入器</t>
+        </is>
+      </c>
+      <c r="J47" s="27" t="inlineStr">
+        <is>
+          <t>无需放第一层</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>images/jayesims-xoxogossipgirlrichtearumors.png</t>
+        </is>
+      </c>
+      <c r="L47" s="28" t="n"/>
+      <c r="M47" s="27" t="inlineStr">
+        <is>
+          <t>游戏玩法</t>
+        </is>
+      </c>
+      <c r="N47" s="29" t="n">
+        <v>46279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Klimter 4 模组（ExtremeTraits/MaliciousTrait/Sunsetlovertrait/PlanetInspiredTraits）模组更新日期改为 2026-09-15
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="G7" s="21" t="n">
-        <v>46225</v>
+        <v>46280</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>46225</v>
@@ -1745,7 +1745,7 @@
         </is>
       </c>
       <c r="G11" s="21" t="n">
-        <v>46216</v>
+        <v>46280</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>46216</v>
@@ -3281,7 +3281,7 @@
         </is>
       </c>
       <c r="G35" s="21" t="n">
-        <v>46255</v>
+        <v>46280</v>
       </c>
       <c r="H35" s="21" t="n">
         <v>46255</v>
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="G40" s="22" t="n">
-        <v>46265</v>
+        <v>46280</v>
       </c>
       <c r="H40" s="22" t="n">
         <v>46265</v>

</xml_diff>

<commit_message>
上新 RBK PregnancyOverhaul_v1.2 怀孕大修（游戏玩法）
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -15,12 +15,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * -#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="_ \¥* #,##0.00_ ;_ \¥* -#,##0.00_ ;_ \¥* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * -#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="168" formatCode="_ \¥* #,##0_ ;_ \¥* -#,##0_ ;_ \¥* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -1031,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="19" min="1" max="1"/>
@@ -4093,6 +4094,68 @@
       </c>
       <c r="N47" s="29" t="n">
         <v>46279</v>
+      </c>
+    </row>
+    <row r="48" ht="36" customHeight="1" s="26">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B48" s="28" t="inlineStr">
+        <is>
+          <t>PregnancyOverhaul_v1.2</t>
+        </is>
+      </c>
+      <c r="C48" s="28" t="inlineStr">
+        <is>
+          <t>怀孕大修</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>RBK</t>
+        </is>
+      </c>
+      <c r="E48" s="28" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/RealismByKatie</t>
+        </is>
+      </c>
+      <c r="F48" s="28" t="inlineStr">
+        <is>
+          <t>https://realismbykatie.com/pregnancy-overhaul/</t>
+        </is>
+      </c>
+      <c r="G48" s="29" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H48" s="29" t="n">
+        <v>46281</v>
+      </c>
+      <c r="I48" s="27" t="inlineStr">
+        <is>
+          <t>Lot51 核心库、XML 注入器</t>
+        </is>
+      </c>
+      <c r="J48" s="27" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>images/rbk-pregnancyoverhaul-v1-2.png</t>
+        </is>
+      </c>
+      <c r="L48" s="28" t="inlineStr"/>
+      <c r="M48" s="27" t="inlineStr">
+        <is>
+          <t>游戏玩法</t>
+        </is>
+      </c>
+      <c r="N48" s="29" t="n">
+        <v>46281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新 JayESims If You’re Wondering If I Hate You… I Absolutely Do 百度网盘下载链接
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -3899,7 +3899,11 @@
           <t>images/jayesims-if-you-re-wondering-if-i-hate-you-i-absolutely-do.png</t>
         </is>
       </c>
-      <c r="L44" s="6" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>链接: https://pan.baidu.com/s/1fmAZJlziQoJjHMbqw7mRBA?pwd=d5zk 提取码: d5zk</t>
+        </is>
+      </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
           <t>游戏玩法</t>

</xml_diff>